<commit_message>
Make this spreadsheet less wrong.
git-svn-id: file:///repo/applications/FRED/branches/mikevdg_importer@44961 976ac4c7-77c1-46cc-9d05-16a3bd20634c
</commit_message>
<xml_diff>
--- a/fred-integration-tests/src/test/resources/importer/paleo.xlsx
+++ b/fred-integration-tests/src/test/resources/importer/paleo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="275">
   <si>
     <t xml:space="preserve">Paleo</t>
   </si>
@@ -862,6 +862,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2402,21 +2403,11 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -2469,10 +2460,18 @@
       <c r="B2" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>1</v>
+      </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
@@ -3870,11 +3869,11 @@
     </row>
   </sheetData>
   <dataValidations count="26">
-    <dataValidation allowBlank="true" operator="lessThanOrEqual" prompt="Enter up to 80 characters here." promptTitle="Enter the locality" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="C1:BA1" type="textLength">
+    <dataValidation allowBlank="true" operator="lessThanOrEqual" prompt="Enter up to 80 characters here." promptTitle="Enter the locality" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="G1:BA1 C2:F2" type="textLength">
       <formula1>80</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="lessThanOrEqual" prompt="Enter up to 80 characters here." promptTitle="Choose a locality." showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="C2:BA2" type="textLength">
+    <dataValidation allowBlank="true" operator="lessThanOrEqual" prompt="Enter up to 80 characters here." promptTitle="Choose a locality." showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="G2:BA2" type="textLength">
       <formula1>80</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>